<commit_message>
chore: update Excel templates for entity status and inside sales
Replaced the existing plantilla_entitystatus.xlsx and plantilla_inside_sales.xlsx files with updated versions to support recent changes in the update scripts. These updates ensure compatibility with the new features and functionalities introduced in the previous commits.
</commit_message>
<xml_diff>
--- a/data/plantilla_inside_sales.xlsx
+++ b/data/plantilla_inside_sales.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\diego_enriquez_idico\idico_projects\rfq\rfq_integration_python\cambios_inside_sales\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\diego_enriquez_idico\idico_projects\actualizacion_insidesales\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB0E28BC-EA6E-47E6-B67C-150AF894A28E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7C4A36F-F8D6-4B29-A154-3C060AD97A39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,22 +20,19 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
   <si>
     <t>id_transaccion</t>
   </si>
   <si>
     <t>id_insidesales</t>
   </si>
-  <si>
-    <t>363zxsa711</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -44,10 +41,9 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
+      <sz val="10"/>
+      <color rgb="FF333333"/>
+      <name val="Carlito"/>
     </font>
   </fonts>
   <fills count="2">
@@ -58,7 +54,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -66,13 +62,38 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="FFE6E6E6"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFE6E6E6"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="FFE6E6E6"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -375,14 +396,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B30"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.85546875" customWidth="1"/>
     <col min="2" max="2" width="22.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" ht="15.75" thickBot="1">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -390,12 +411,236 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" ht="15.75" thickBot="1">
       <c r="A2" s="1">
-        <v>1240659</v>
-      </c>
-      <c r="B2" t="s">
-        <v>2</v>
+        <v>1249706</v>
+      </c>
+      <c r="B2">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="15.75" thickBot="1">
+      <c r="A3" s="1">
+        <v>1254179</v>
+      </c>
+      <c r="B3">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="15.75" thickBot="1">
+      <c r="A4" s="1">
+        <v>1283268</v>
+      </c>
+      <c r="B4">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="15.75" thickBot="1">
+      <c r="A5" s="1">
+        <v>1320003</v>
+      </c>
+      <c r="B5">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="15.75" thickBot="1">
+      <c r="A6" s="1">
+        <v>1289200</v>
+      </c>
+      <c r="B6">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="15.75" thickBot="1">
+      <c r="A7" s="1">
+        <v>1283269</v>
+      </c>
+      <c r="B7">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="15.75" thickBot="1">
+      <c r="A8" s="1">
+        <v>1283778</v>
+      </c>
+      <c r="B8">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="15.75" thickBot="1">
+      <c r="A9" s="1">
+        <v>1288792</v>
+      </c>
+      <c r="B9">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="15.75" thickBot="1">
+      <c r="A10" s="1">
+        <v>1285824</v>
+      </c>
+      <c r="B10">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="15.75" thickBot="1">
+      <c r="A11" s="1">
+        <v>1285014</v>
+      </c>
+      <c r="B11">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="15.75" thickBot="1">
+      <c r="A12" s="1">
+        <v>1319802</v>
+      </c>
+      <c r="B12">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="15.75" thickBot="1">
+      <c r="A13" s="1">
+        <v>1285316</v>
+      </c>
+      <c r="B13">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="15.75" thickBot="1">
+      <c r="A14" s="1">
+        <v>1320104</v>
+      </c>
+      <c r="B14">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="15.75" thickBot="1">
+      <c r="A15" s="1">
+        <v>1308492</v>
+      </c>
+      <c r="B15">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" ht="15.75" thickBot="1">
+      <c r="A16" s="1">
+        <v>1285116</v>
+      </c>
+      <c r="B16">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="15.75" thickBot="1">
+      <c r="A17" s="1">
+        <v>1288384</v>
+      </c>
+      <c r="B17">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="15.75" thickBot="1">
+      <c r="A18" s="1">
+        <v>1289103</v>
+      </c>
+      <c r="B18">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="15.75" thickBot="1">
+      <c r="A19" s="1">
+        <v>1309399</v>
+      </c>
+      <c r="B19">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="15.75" thickBot="1">
+      <c r="A20" s="1">
+        <v>1308293</v>
+      </c>
+      <c r="B20">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" thickBot="1">
+      <c r="A21" s="1">
+        <v>1296431</v>
+      </c>
+      <c r="B21">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" thickBot="1">
+      <c r="A22" s="1">
+        <v>1309394</v>
+      </c>
+      <c r="B22">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" thickBot="1">
+      <c r="A23" s="1">
+        <v>1295926</v>
+      </c>
+      <c r="B23">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" thickBot="1">
+      <c r="A24" s="1">
+        <v>1308488</v>
+      </c>
+      <c r="B24">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" thickBot="1">
+      <c r="A25" s="1">
+        <v>1308284</v>
+      </c>
+      <c r="B25">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="15.75" thickBot="1">
+      <c r="A26" s="1">
+        <v>1312479</v>
+      </c>
+      <c r="B26">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" ht="15.75" thickBot="1">
+      <c r="A27" s="1">
+        <v>1314497</v>
+      </c>
+      <c r="B27">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" ht="15.75" thickBot="1">
+      <c r="A28" s="1">
+        <v>1315519</v>
+      </c>
+      <c r="B28">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" ht="15.75" thickBot="1">
+      <c r="A29" s="1">
+        <v>1316230</v>
+      </c>
+      <c r="B29">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2">
+      <c r="A30" s="2">
+        <v>1316234</v>
+      </c>
+      <c r="B30">
+        <v>361</v>
       </c>
     </row>
   </sheetData>

</xml_diff>